<commit_message>
fix some streaming files
</commit_message>
<xml_diff>
--- a/streaming/oportunidades.xlsx
+++ b/streaming/oportunidades.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,108 +453,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>902dc150-137b-450a-b9e9-7efa9f5fdff5</t>
+          <t>a55bb759-bb9d-4c7f-8bac-41fc6c6a9069</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>209662.6</v>
+        <v>63176.49</v>
       </c>
       <c r="C2" t="n">
-        <v>675230.4375</v>
+        <v>314537.59375</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-08-14 15:15:40</t>
+          <t>2025-08-17 23:23:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0edd5161-d4bc-4910-9e42-9d1309e15e31</t>
+          <t>a202b2a3-8cd4-49f9-8fe6-63c3278fc417</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>247728.46</v>
+        <v>130979.72</v>
       </c>
       <c r="C3" t="n">
-        <v>278337.78125</v>
+        <v>440479.875</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-08-14 15:15:45</t>
+          <t>2025-08-17 23:23:25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>98c9e861-3f12-4735-a7f9-b319198b6b38</t>
+          <t>517b23e2-f4b2-49b0-ba0c-7252e12b0cb9</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>87549.91</v>
+        <v>183699.98</v>
       </c>
       <c r="C4" t="n">
-        <v>207457.625</v>
+        <v>352367.8125</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-08-14 15:15:51</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>75270875-d924-4562-966e-4fc5bb5dafd5</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>212953.51</v>
-      </c>
-      <c r="C5" t="n">
-        <v>429066.28125</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2025-08-14 15:15:54</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>48526674-4a35-463b-83a0-d81d12427bbd</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>188027.28</v>
-      </c>
-      <c r="C6" t="n">
-        <v>460065.75</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2025-08-14 15:15:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>13a9d369-2f90-4993-a6c2-e28e276fa735</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>134571.15</v>
-      </c>
-      <c r="C7" t="n">
-        <v>314840.3125</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2025-08-14 15:16:02</t>
+          <t>2025-08-17 23:23:28</t>
         </is>
       </c>
     </row>

</xml_diff>